<commit_message>
Adicionado banner a vista
</commit_message>
<xml_diff>
--- a/promocoes.xlsx
+++ b/promocoes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael Castro\Documents\gerar-imagem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FA30E3-0B9B-429D-9F8F-2AA0B51BCC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7927C9CE-67EE-454A-80B4-B42450CA1AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{E5CF45C3-0614-48A6-8C4F-006EC199C177}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>descricao</t>
   </si>
@@ -42,10 +42,130 @@
     <t>valor_original</t>
   </si>
   <si>
-    <t>42.0042</t>
-  </si>
-  <si>
     <t>PATINS MTB VB CH10 POWER 70MM</t>
+  </si>
+  <si>
+    <t>12.0062</t>
+  </si>
+  <si>
+    <t>70.0011</t>
+  </si>
+  <si>
+    <t>46.0043</t>
+  </si>
+  <si>
+    <t>46.0042</t>
+  </si>
+  <si>
+    <t>15.0121</t>
+  </si>
+  <si>
+    <t>44.0010</t>
+  </si>
+  <si>
+    <t>20.0001</t>
+  </si>
+  <si>
+    <t>44.0041</t>
+  </si>
+  <si>
+    <t>04.0120</t>
+  </si>
+  <si>
+    <t>03.0099</t>
+  </si>
+  <si>
+    <t>07.0087</t>
+  </si>
+  <si>
+    <t>15.0124</t>
+  </si>
+  <si>
+    <t>04.0062</t>
+  </si>
+  <si>
+    <t>04.0212</t>
+  </si>
+  <si>
+    <t>23.0130</t>
+  </si>
+  <si>
+    <t>04.0177</t>
+  </si>
+  <si>
+    <t>04.0189</t>
+  </si>
+  <si>
+    <t>23.0128</t>
+  </si>
+  <si>
+    <t>23.0127</t>
+  </si>
+  <si>
+    <t>04.0135</t>
+  </si>
+  <si>
+    <t>21.0067</t>
+  </si>
+  <si>
+    <t>KIT 2X9 SHIMANO ALIVIO   FREIO HIDRAULICO MT200 - CUBO 32F</t>
+  </si>
+  <si>
+    <t>LIMPEZA GERAL SOLIFES 500ML</t>
+  </si>
+  <si>
+    <t>PATINS MTB VB ORBITAL 70MM GTS (BLISTER)</t>
+  </si>
+  <si>
+    <t>RODA LIVRE 20D COMANDER</t>
+  </si>
+  <si>
+    <t>GARFO 26 S. 21.1 MODE PTO</t>
+  </si>
+  <si>
+    <t>PEDIV 165MM R CICLO CROM</t>
+  </si>
+  <si>
+    <t>GARFO 29 S. AH SET ACO TAIWAN PTO</t>
+  </si>
+  <si>
+    <t>SELIM BEACH 2M INVIKTUS PTO C/ REFLETOR</t>
+  </si>
+  <si>
+    <t>CAMARA 26 BUTIL BISON (CAIXA FECHADA)</t>
+  </si>
+  <si>
+    <t>PASTILHA REFIL GTS QUAD. C/MOLA F DISCO PAR (GRANEL)</t>
+  </si>
+  <si>
+    <t>RODA LIVRE 7V INDEX FALCON 14/28 BRONZE</t>
+  </si>
+  <si>
+    <t>SELIM MTB VAZ INVIKTUS PTO</t>
+  </si>
+  <si>
+    <t>SELIM MTB VAZ GTS HY-298 NEO PTO</t>
+  </si>
+  <si>
+    <t>MANOPLA FREERIDE MOOVE VERMELHO 165MM C/ FLANGE</t>
+  </si>
+  <si>
+    <t>SELIM MTB NITRUS BELUGA C/CAR PTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SELIM BEACH 2M LTX186-1 PTO C/CAR </t>
+  </si>
+  <si>
+    <t>MANOPLA FREERIDE MOOVE LARANJA 165MM C/ FLANGE</t>
+  </si>
+  <si>
+    <t>MANOPLA FREERIDE MOOVE ROSA 165MM C/ FLANGE</t>
+  </si>
+  <si>
+    <t>SELIM SRX HAVAC VAZ R CICLO PTO</t>
+  </si>
+  <si>
+    <t>CUBO D/T AL ROLLER VIPER PTO</t>
   </si>
 </sst>
 </file>
@@ -70,10 +190,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF333333"/>
-      <name val="Segoe UI"/>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -99,16 +221,16 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A8FE7EE-E501-4B97-88C7-40543CDDBCF9}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76.140625" bestFit="1" customWidth="1"/>
@@ -446,99 +568,299 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5">
+        <v>1138</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1115.24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="5">
+        <v>15.42</v>
+      </c>
+      <c r="D3" s="5">
+        <v>14.9574</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1.3871</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3">
-        <v>2.21</v>
-      </c>
-      <c r="D2" s="2">
-        <v>2.13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="2"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="2"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="2"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="2"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.2138999999999998</v>
+      </c>
+      <c r="D5" s="5">
+        <v>2.1253439999999997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5">
+        <v>5.9735999999999994</v>
+      </c>
+      <c r="D6" s="5">
+        <v>5.7346559999999993</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="5">
+        <v>51.92</v>
+      </c>
+      <c r="D7" s="5">
+        <v>49.843200000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="5">
+        <v>16.989999999999998</v>
+      </c>
+      <c r="D8" s="5">
+        <v>16.310399999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="5">
+        <v>48.59</v>
+      </c>
+      <c r="D9" s="5">
+        <v>46.6464</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="5">
+        <v>23.82</v>
+      </c>
+      <c r="D10" s="5">
+        <v>22.8672</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="5">
+        <v>6.99</v>
+      </c>
+      <c r="D11" s="5">
+        <v>6.5009700000000006</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="5">
+        <v>1.9649999999999999</v>
+      </c>
+      <c r="D12" s="5">
+        <v>1.8274499999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="5">
+        <v>22.008000000000003</v>
+      </c>
+      <c r="D13" s="5">
+        <v>20.247360000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="5">
+        <v>23.841999999999999</v>
+      </c>
+      <c r="D14" s="5">
+        <v>21.934639999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="5">
+        <v>19.623799999999999</v>
+      </c>
+      <c r="D15" s="5">
+        <v>18.053895999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="5">
+        <v>7.5979999999999999</v>
+      </c>
+      <c r="D16" s="5">
+        <v>6.9901599999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="5">
+        <v>19.623799999999999</v>
+      </c>
+      <c r="D17" s="5">
+        <v>18.053895999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="5">
+        <v>41.278100000000002</v>
+      </c>
+      <c r="D18" s="5">
+        <v>37.975852000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="5">
+        <v>7.5979999999999999</v>
+      </c>
+      <c r="D19" s="5">
+        <v>6.9901599999999995</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="5">
+        <v>7.5979999999999999</v>
+      </c>
+      <c r="D20" s="5">
+        <v>6.9901599999999995</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="5">
+        <v>74.997500000000002</v>
+      </c>
+      <c r="D21" s="5">
+        <v>68.997700000000009</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="5">
+        <v>34.06</v>
+      </c>
+      <c r="D22" s="5">
+        <v>31.3352</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D18" xr:uid="{0A8FE7EE-E501-4B97-88C7-40543CDDBCF9}"/>

</xml_diff>